<commit_message>
Move amortization property block right
</commit_message>
<xml_diff>
--- a/Project Rooms/Amortization/templates/Buyer-Facing Amortization Chart Template.xlsx
+++ b/Project Rooms/Amortization/templates/Buyer-Facing Amortization Chart Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Codex\Wiki Files\Project Rooms\Amortization\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E85C4A58-3682-4DB1-B836-D4956B20B09C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E8FB4BA-B07A-4ABB-9FB6-156DD7715D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{06CA6E75-7099-4174-99F2-A983CB5A5C31}"/>
   </bookViews>
@@ -218,20 +218,8 @@
   <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -249,6 +237,18 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -597,374 +597,374 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="4"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
+      <c r="A2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7" t="s">
+      <c r="B3" s="13"/>
+      <c r="C3" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="6" t="s">
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="14"/>
+      <c r="I3" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7" t="s">
+      <c r="B4" s="13"/>
+      <c r="C4" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="6" t="s">
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="14"/>
+      <c r="I4" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
+      <c r="J4" s="14"/>
+      <c r="K4" s="14"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7" t="s">
+      <c r="B5" s="13"/>
+      <c r="C5" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="6" t="s">
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="14"/>
+      <c r="I5" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="14"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7" t="s">
+      <c r="B6" s="13"/>
+      <c r="C6" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="6" t="s">
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="14"/>
+      <c r="I6" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
+      <c r="A7" s="2"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
     </row>
     <row r="8" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H8" s="8" t="s">
+      <c r="H8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="I8" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="K8" s="8" t="s">
+      <c r="K8" s="4" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="10"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
+      <c r="A9" s="6"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="10"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12"/>
-      <c r="K10" s="12"/>
+      <c r="A10" s="6"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="10"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="10"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="12"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="10"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="12"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="10"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="12"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="10"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="12"/>
+      <c r="A15" s="6"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="10"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="12"/>
-      <c r="J16" s="12"/>
-      <c r="K16" s="12"/>
+      <c r="A16" s="6"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="10"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
-      <c r="I17" s="12"/>
-      <c r="J17" s="12"/>
-      <c r="K17" s="12"/>
+      <c r="A17" s="6"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="10"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12"/>
+      <c r="A18" s="6"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="8"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="10"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
-      <c r="K19" s="12"/>
+      <c r="A19" s="6"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="8"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="10"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="12"/>
-      <c r="J20" s="12"/>
-      <c r="K20" s="12"/>
+      <c r="A20" s="6"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="8"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="15">
-        <f>SUM(E9:E20)</f>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="11">
+        <f t="shared" ref="E21:J21" si="0">SUM(E9:E20)</f>
         <v>0</v>
       </c>
-      <c r="F21" s="15">
-        <f>SUM(F9:F20)</f>
+      <c r="F21" s="11">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G21" s="15">
-        <f>SUM(G9:G20)</f>
+      <c r="G21" s="11">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H21" s="15">
-        <f>SUM(H9:H20)</f>
+      <c r="H21" s="11">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I21" s="15">
-        <f>SUM(I9:I20)</f>
+      <c r="I21" s="11">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J21" s="15">
-        <f>SUM(J9:J20)</f>
+      <c r="J21" s="11">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K21" s="16"/>
+      <c r="K21" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A21:D21"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:K5"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="I5:K5"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="I6:K6"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C3:F3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="I3:K3"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:K4"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:K3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:K4"/>
+    <mergeCell ref="A21:D21"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="4800" verticalDpi="4800" r:id="rId1"/>

</xml_diff>

<commit_message>
Preserve Amortization appendix row
</commit_message>
<xml_diff>
--- a/Project Rooms/Amortization/templates/Buyer-Facing Amortization Chart Template.xlsx
+++ b/Project Rooms/Amortization/templates/Buyer-Facing Amortization Chart Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Codex\Wiki Files\Project Rooms\Amortization\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E8FB4BA-B07A-4ABB-9FB6-156DD7715D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDFF8F7F-7BDF-4338-95C8-D6B0189B1B30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{06CA6E75-7099-4174-99F2-A983CB5A5C31}"/>
   </bookViews>
@@ -16,9 +16,9 @@
     <sheet name="12 Month Chart" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'12 Month Chart'!$A$1:$K$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'12 Month Chart'!$A$2:$K$22</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterate="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>{{PROJECT}} - 12 Month Amortization Chart</t>
   </si>
@@ -129,15 +129,20 @@
   </si>
   <si>
     <t>Totals for displayed 12-month period</t>
+  </si>
+  <si>
+    <t>Appendix "A"</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.000%"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="167" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -215,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -236,18 +241,30 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -586,188 +603,191 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.7109375" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" style="1" customWidth="1"/>
-    <col min="3" max="9" width="10.7109375" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" customWidth="1"/>
+    <col min="4" max="9" width="10.7109375" customWidth="1"/>
     <col min="10" max="10" width="11.7109375" customWidth="1"/>
     <col min="11" max="11" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+    </row>
+    <row r="2" spans="1:11" ht="21" x14ac:dyDescent="0.35">
+      <c r="A2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="2"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="14" t="s">
+      <c r="B4" s="14"/>
+      <c r="C4" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="13" t="s">
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14" t="s">
+      <c r="H4" s="16"/>
+      <c r="I4" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="J4" s="16"/>
+      <c r="K4" s="16"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="13"/>
-      <c r="C4" s="14" t="s">
+      <c r="B5" s="14"/>
+      <c r="C5" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="13" t="s">
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14" t="s">
+      <c r="H5" s="16"/>
+      <c r="I5" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="14" t="s">
+      <c r="B6" s="14"/>
+      <c r="C6" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="13" t="s">
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14" t="s">
+      <c r="H6" s="16"/>
+      <c r="I6" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="14" t="s">
+      <c r="B7" s="14"/>
+      <c r="C7" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="13" t="s">
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14" t="s">
+      <c r="H7" s="16"/>
+      <c r="I7" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="14"/>
-      <c r="K6" s="14"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-    </row>
-    <row r="8" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="J7" s="20"/>
+      <c r="K7" s="20"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+    </row>
+    <row r="9" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E9" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F9" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H9" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="I9" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="J9" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="K9" s="4" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="6"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="8"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="6"/>
@@ -913,41 +933,63 @@
       <c r="K20" s="8"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="6"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="12"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="11">
-        <f t="shared" ref="E21:J21" si="0">SUM(E9:E20)</f>
+      <c r="B22" s="15"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="11">
+        <f t="shared" ref="E22:J22" si="0">SUM(E10:E21)</f>
         <v>0</v>
       </c>
-      <c r="F21" s="11">
+      <c r="F22" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G21" s="11">
+      <c r="G22" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H21" s="11">
+      <c r="H22" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I21" s="11">
+      <c r="I22" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J21" s="11">
+      <c r="J22" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K21" s="10"/>
+      <c r="K22" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="19">
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A22:D22"/>
     <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:K4"/>
     <mergeCell ref="C5:F5"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="I5:K5"/>
@@ -955,16 +997,8 @@
     <mergeCell ref="C6:F6"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="I6:K6"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C3:F3"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="I3:K3"/>
-    <mergeCell ref="C4:F4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="I4:K4"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:F7"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="4800" verticalDpi="4800" r:id="rId1"/>

</xml_diff>